<commit_message>
Debugged version of Step-by-step adjust object position to survey data XY or XYZ.
</commit_message>
<xml_diff>
--- a/NO-BN/Lua/Scripts/FE/Object positioning/Step-by-step - Adjust objects to XY(Z) from Excel/Tiny survey data example adjustment coordinates).xlsx
+++ b/NO-BN/Lua/Scripts/FE/Object positioning/Step-by-step - Adjust objects to XY(Z) from Excel/Tiny survey data example adjustment coordinates).xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\claus\Documents\GitHub\RailCOMPLETE-DNA-NO-BN\NO-BN\Lua\Scripts\FE\Object positioning\Step-by-step - Adjust objects to XY(Z) from Excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{98F9E92C-C465-48E1-B30F-E5ADF3427638}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{020A6C4C-F017-41C9-A564-CF473996C866}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="12255" yWindow="4935" windowWidth="18225" windowHeight="14310" xr2:uid="{458BF04D-148A-4D8F-8462-62E87D0FA389}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="12">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="13" uniqueCount="13">
   <si>
     <t>X</t>
   </si>
@@ -72,6 +72,9 @@
   </si>
   <si>
     <t>Terte</t>
+  </si>
+  <si>
+    <t>Nr</t>
   </si>
 </sst>
 </file>
@@ -452,104 +455,125 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C7DE9C06-F12D-430F-80BA-DA374A76F7E0}">
-  <dimension ref="A1:D7"/>
+  <dimension ref="A1:E7"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="23.42578125" customWidth="1"/>
+    <col min="2" max="2" width="23.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="C1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="D1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="E1" s="1" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2">
+        <v>1</v>
+      </c>
+      <c r="B2" t="s">
         <v>2</v>
       </c>
-      <c r="B2">
+      <c r="C2">
         <v>94.2</v>
       </c>
-      <c r="C2">
+      <c r="D2">
         <v>76.64</v>
       </c>
-      <c r="D2">
+      <c r="E2">
         <v>1.1000000000000001</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A3">
+        <v>2</v>
+      </c>
+      <c r="B3" t="s">
         <v>8</v>
       </c>
-      <c r="B3" t="s">
+      <c r="C3" t="s">
         <v>4</v>
       </c>
-      <c r="C3">
+      <c r="D3">
         <v>123.4</v>
       </c>
-      <c r="D3">
-        <v>5.5</v>
-      </c>
-    </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
+      <c r="E3">
+        <v>2.2000000000000002</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A4">
+        <v>3</v>
+      </c>
+      <c r="B4" t="s">
         <v>6</v>
       </c>
-      <c r="B4">
+      <c r="C4">
         <v>88.95</v>
       </c>
-      <c r="C4">
+      <c r="D4">
         <v>123.35</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A5">
+        <v>4</v>
+      </c>
+      <c r="B5" t="s">
         <v>7</v>
       </c>
-      <c r="B5">
+      <c r="C5">
         <v>98.27</v>
       </c>
-      <c r="C5">
+      <c r="D5">
         <v>159.51</v>
       </c>
-      <c r="D5">
+      <c r="E5">
         <v>3.3</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A6">
+        <v>5</v>
+      </c>
+      <c r="B6" t="s">
         <v>9</v>
       </c>
-      <c r="B6">
+      <c r="C6">
         <v>92.1</v>
       </c>
-      <c r="C6">
+      <c r="D6">
         <v>128.69999999999999</v>
       </c>
-      <c r="D6" t="s">
+      <c r="E6" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A7" t="s">
+    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A7">
+        <v>6</v>
+      </c>
+      <c r="B7" t="s">
         <v>11</v>
       </c>
-      <c r="B7">
+      <c r="C7">
         <v>100.32</v>
       </c>
-      <c r="C7">
+      <c r="D7">
         <v>204.81</v>
       </c>
-      <c r="D7">
+      <c r="E7">
         <v>4.4000000000000004</v>
       </c>
     </row>

</xml_diff>